<commit_message>
V1.2.1 Ajout du support des cartes multifaces
</commit_message>
<xml_diff>
--- a/Base_Reference.xlsx
+++ b/Base_Reference.xlsx
@@ -2580,6 +2580,11 @@
           <t>Peter Parker // Amazing Spider-Man</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Peter Parker // L'incroyable Spider-Man</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>peterparkeramazingspiderman</t>
@@ -2611,6 +2616,16 @@
       <c r="N11" t="inlineStr">
         <is>
           <t>Human;Scientist;Hero;//;Legendary;Creature</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>--- Peter Parker ---
+Quand Peter Parker arrive, créez un jeton de créature 2/1 verte Araignée avec la portée.
+{1}{G}{W}{U} : Transformez Peter Parker. N'activez que lorsque vous pourriez lancer un rituel.
+--- L'incroyable Spider-Man ---
+Vigilance, portée
+Chaque sort légendaire que vous lancez qui a au moins une couleur a lanceur de toile {G}{W}{U}. (Vous pouvez lancer un sort pour son coût de lanceur de toile si vous renvoyez aussi une créature engagée que vous contrôlez dans la main de son propriétaire.)</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -8387,6 +8402,11 @@
           <t>Norman Osborn // Green Goblin</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Norman Osborn // Bouffon vert</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>normanosborngreengoblin</t>
@@ -8418,6 +8438,18 @@
       <c r="N40" t="inlineStr">
         <is>
           <t>Human;Scientist;Villain;//;Legendary;Creature</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>--- Norman Osborn ---
+Norman Osborn ne peut pas être bloqué.
+À chaque fois que Norman Osborn inflige des blessures de combat à un joueur, il connive. (Piochez une carte, puis défaussez-vous d'une carte. Si vous vous êtes défaussé d'une carte non-terrain, mettez un marqueur +1/+1 sur cette créature.)
+{1}{U}{B}{R} : Transformez Norman Osborn. N'activez que lorsque vous pourriez lancer un rituel.
+--- Bouffon vert ---
+Vol, menace
+Les sorts que vous lancez depuis votre cimetière coûtent {2} de moins à lancer.
+Formule du bouffon - Chaque carte non-terrain dans votre cimetière a le désordre. Le coût de désordre est égal à son coût de mana. (Vous pouvez lancer une carte depuis votre cimetière pour son coût de désordre si vous vous en êtes défaussé ce tour-ci. Les règles de restriction de temps s'appliquent quand même.)</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -11536,6 +11568,11 @@
           <t>Eddie Brock // Venom, Lethal Protector</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Eddie Brock // Venom, protecteur mortel</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>eddiebrockvenomlethalprotector</t>
@@ -11567,6 +11604,16 @@
       <c r="N56" t="inlineStr">
         <is>
           <t>Human;Hero;Villain;//;Legendary;Creature</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>--- Eddie Brock ---
+Quand Eddie Brock arrive, renvoyez sur le champ de bataille une carte de créature ciblée avec une valeur de mana inférieure ou égale à 1 depuis votre cimetière.
+{3}{B}{R}{G} : Transformez Eddie Brock. N'activez que lorsque vous pourriez lancer un rituel.
+--- Venom, protecteur mortel ---
+Menace, piétinement, célérité
+À chaque fois que Venom attaque, vous pouvez sacrifier une autre créature. Si vous faites ainsi, piochez X cartes, puis vous pouvez mettre sur le champ de bataille, depuis votre main, une carte de permanent avec une valeur de mana inférieure ou égale à X, X étant la valeur de mana de la créature sacrifiée.</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -16142,6 +16189,11 @@
           <t>Gwen Stacy // Ghost-Spider</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Gwen Stacy // Ghost-Spider</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>gwenstacyghostspider</t>
@@ -16173,6 +16225,17 @@
       <c r="N79" t="inlineStr">
         <is>
           <t>Human;Performer;Hero;//;Legendary;Creature</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>--- Gwen Stacy ---
+Quand Gwen Stacy arrive, exilez la carte du dessus de votre bibliothèque. Vous pouvez jouer cette carte tant que vous contrôlez cette créature.
+{2}{U}{R}{W} : Transformez Gwen Stacy. N'activez que lorsque vous pourriez lancer un rituel.
+--- Ghost-Spider ---
+Vol, vigilance, célérité
+À chaque fois que vous jouez un terrain depuis l'exil ou que vous lancez un sort depuis l'exil, mettez un marqueur +1/+1 sur Ghost-Spider.
+Retirez deux marqueurs de Ghost-Spider : Exilez la carte du dessus de votre bibliothèque. Vous pouvez jouer cette carte ce tour-ci.</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -22194,6 +22257,11 @@
           <t>Miles Morales // Ultimate Spider-Man</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Miles Morales // L'ultime Spider-Man</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
           <t>milesmoralesultimatespiderman</t>
@@ -22225,6 +22293,17 @@
       <c r="N109" t="inlineStr">
         <is>
           <t>Human;Citizen;Hero;//;Legendary;Creature</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>--- Miles Morales ---
+Quand Miles Morales arrive, ciblez jusqu'à deux créatures. Mettez un marqueur +1/+1 sur chacune d'elles.
+{3}{R}{G}{W} : Transformez Miles Morales. N'activez que lorsque vous pourriez lancer un rituel.
+--- L'ultime Spider-Man ---
+Initiative, célérité
+Camouflage - {2} : Mettez un marqueur +1/+1 sur L'ultime Spider-Man. Il acquiert la défense talismanique et devient incolore jusqu'à la fin du tour.
+À chaque fois que vous attaquez, doublez le nombre de chaque sorte de marqueur sur chaque araignée et sur chaque créature légendaire que vous contrôlez.</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">

</xml_diff>